<commit_message>
updated environmental data and script updates
</commit_message>
<xml_diff>
--- a/2026/data/GOA_arrowtooth_2026.xlsx
+++ b/2026/data/GOA_arrowtooth_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kalei.shotwell\Work\GitHub\GOA-ATF-ESP\2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230A647E-B345-4440-A44E-751A718EBD6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C594D3-7AC1-436B-A3F8-C9E33CD4242E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="7" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1298" uniqueCount="500">
   <si>
     <t>Sheet name</t>
   </si>
@@ -1550,9 +1550,6 @@
     <t>Diet_comp_weights</t>
   </si>
   <si>
-    <t>BTempC</t>
-  </si>
-  <si>
     <t>...25</t>
   </si>
   <si>
@@ -1578,6 +1575,39 @@
   </si>
   <si>
     <t>Stomach_proportion_by_weight</t>
+  </si>
+  <si>
+    <t>pred</t>
+  </si>
+  <si>
+    <t>sst</t>
+  </si>
+  <si>
+    <t>larvae</t>
+  </si>
+  <si>
+    <t>eke_east</t>
+  </si>
+  <si>
+    <t>eke_west</t>
+  </si>
+  <si>
+    <t>copepods</t>
+  </si>
+  <si>
+    <t>cond</t>
+  </si>
+  <si>
+    <t>nearshore_age1</t>
+  </si>
+  <si>
+    <t>euph</t>
+  </si>
+  <si>
+    <t>bt</t>
+  </si>
+  <si>
+    <t>lg_copepods</t>
   </si>
 </sst>
 </file>
@@ -5295,375 +5325,1907 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>153</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+        <v>489</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2">
+        <v>1977</v>
+      </c>
+      <c r="B2">
+        <v>15248.38631</v>
+      </c>
+      <c r="C2" t="s">
+        <v>478</v>
+      </c>
+      <c r="D2" t="s">
+        <v>478</v>
+      </c>
+      <c r="E2" t="s">
+        <v>478</v>
+      </c>
+      <c r="F2" t="s">
+        <v>478</v>
+      </c>
+      <c r="G2" t="s">
+        <v>478</v>
+      </c>
+      <c r="H2" t="s">
+        <v>478</v>
+      </c>
+      <c r="I2" t="s">
+        <v>478</v>
+      </c>
+      <c r="J2" t="s">
+        <v>478</v>
+      </c>
+      <c r="K2" t="s">
+        <v>478</v>
+      </c>
+      <c r="L2" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1978</v>
+      </c>
+      <c r="B3">
+        <v>13659.28636</v>
+      </c>
+      <c r="C3" t="s">
+        <v>478</v>
+      </c>
+      <c r="D3" t="s">
+        <v>478</v>
+      </c>
+      <c r="E3" t="s">
+        <v>478</v>
+      </c>
+      <c r="F3" t="s">
+        <v>478</v>
+      </c>
+      <c r="G3" t="s">
+        <v>478</v>
+      </c>
+      <c r="H3" t="s">
+        <v>478</v>
+      </c>
+      <c r="I3" t="s">
+        <v>478</v>
+      </c>
+      <c r="J3" t="s">
+        <v>478</v>
+      </c>
+      <c r="K3" t="s">
+        <v>478</v>
+      </c>
+      <c r="L3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>1979</v>
       </c>
-      <c r="B2">
-        <v>4.91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3">
+      <c r="B4">
+        <v>13105.91462</v>
+      </c>
+      <c r="C4" t="s">
+        <v>478</v>
+      </c>
+      <c r="D4" t="s">
+        <v>478</v>
+      </c>
+      <c r="E4" t="s">
+        <v>478</v>
+      </c>
+      <c r="F4" t="s">
+        <v>478</v>
+      </c>
+      <c r="G4" t="s">
+        <v>478</v>
+      </c>
+      <c r="H4" t="s">
+        <v>478</v>
+      </c>
+      <c r="I4" t="s">
+        <v>478</v>
+      </c>
+      <c r="J4" t="s">
+        <v>478</v>
+      </c>
+      <c r="K4" t="s">
+        <v>478</v>
+      </c>
+      <c r="L4" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>1980</v>
       </c>
-      <c r="B3">
-        <v>5.03</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4">
+      <c r="B5">
+        <v>12645.50397</v>
+      </c>
+      <c r="C5" t="s">
+        <v>478</v>
+      </c>
+      <c r="D5" t="s">
+        <v>478</v>
+      </c>
+      <c r="E5" t="s">
+        <v>478</v>
+      </c>
+      <c r="F5" t="s">
+        <v>478</v>
+      </c>
+      <c r="G5" t="s">
+        <v>478</v>
+      </c>
+      <c r="H5" t="s">
+        <v>478</v>
+      </c>
+      <c r="I5" t="s">
+        <v>478</v>
+      </c>
+      <c r="J5" t="s">
+        <v>478</v>
+      </c>
+      <c r="K5" t="s">
+        <v>478</v>
+      </c>
+      <c r="L5" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>1981</v>
       </c>
-      <c r="B4">
-        <v>5.71</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5">
+      <c r="B6">
+        <v>12943.0841</v>
+      </c>
+      <c r="C6" t="s">
+        <v>478</v>
+      </c>
+      <c r="D6">
+        <v>-1.145475104</v>
+      </c>
+      <c r="E6" t="s">
+        <v>478</v>
+      </c>
+      <c r="F6" t="s">
+        <v>478</v>
+      </c>
+      <c r="G6" t="s">
+        <v>478</v>
+      </c>
+      <c r="H6" t="s">
+        <v>478</v>
+      </c>
+      <c r="I6" t="s">
+        <v>478</v>
+      </c>
+      <c r="J6" t="s">
+        <v>478</v>
+      </c>
+      <c r="K6" t="s">
+        <v>478</v>
+      </c>
+      <c r="L6" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7">
         <v>1982</v>
       </c>
-      <c r="B5">
+      <c r="B7">
+        <v>10594.435020000001</v>
+      </c>
+      <c r="C7" t="s">
+        <v>478</v>
+      </c>
+      <c r="D7">
+        <v>-1.8218033179999999</v>
+      </c>
+      <c r="E7" t="s">
+        <v>478</v>
+      </c>
+      <c r="F7" t="s">
+        <v>478</v>
+      </c>
+      <c r="G7" t="s">
+        <v>478</v>
+      </c>
+      <c r="H7" t="s">
+        <v>478</v>
+      </c>
+      <c r="I7" t="s">
+        <v>478</v>
+      </c>
+      <c r="J7" t="s">
+        <v>478</v>
+      </c>
+      <c r="K7" t="s">
+        <v>478</v>
+      </c>
+      <c r="L7" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1983</v>
+      </c>
+      <c r="B8">
+        <v>11659.27455</v>
+      </c>
+      <c r="C8" t="s">
+        <v>478</v>
+      </c>
+      <c r="D8">
+        <v>-0.968959299</v>
+      </c>
+      <c r="E8" t="s">
+        <v>478</v>
+      </c>
+      <c r="F8" t="s">
+        <v>478</v>
+      </c>
+      <c r="G8" t="s">
+        <v>478</v>
+      </c>
+      <c r="H8" t="s">
+        <v>478</v>
+      </c>
+      <c r="I8" t="s">
+        <v>478</v>
+      </c>
+      <c r="J8" t="s">
+        <v>478</v>
+      </c>
+      <c r="K8" t="s">
+        <v>478</v>
+      </c>
+      <c r="L8" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1984</v>
+      </c>
+      <c r="B9">
+        <v>13151.98849</v>
+      </c>
+      <c r="C9" t="s">
+        <v>478</v>
+      </c>
+      <c r="D9" t="s">
+        <v>478</v>
+      </c>
+      <c r="E9" t="s">
+        <v>478</v>
+      </c>
+      <c r="F9" t="s">
+        <v>478</v>
+      </c>
+      <c r="G9" t="s">
+        <v>478</v>
+      </c>
+      <c r="H9" t="s">
+        <v>478</v>
+      </c>
+      <c r="I9" t="s">
+        <v>478</v>
+      </c>
+      <c r="J9" t="s">
+        <v>478</v>
+      </c>
+      <c r="K9" t="s">
+        <v>478</v>
+      </c>
+      <c r="L9" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1985</v>
+      </c>
+      <c r="B10">
+        <v>21351.045409999999</v>
+      </c>
+      <c r="C10">
+        <v>4.29</v>
+      </c>
+      <c r="D10">
+        <v>1.7271244160000001</v>
+      </c>
+      <c r="E10" t="s">
+        <v>478</v>
+      </c>
+      <c r="F10" t="s">
+        <v>478</v>
+      </c>
+      <c r="G10" t="s">
+        <v>478</v>
+      </c>
+      <c r="H10" t="s">
+        <v>478</v>
+      </c>
+      <c r="I10" t="s">
+        <v>478</v>
+      </c>
+      <c r="J10" t="s">
+        <v>478</v>
+      </c>
+      <c r="K10" t="s">
+        <v>478</v>
+      </c>
+      <c r="L10" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1986</v>
+      </c>
+      <c r="B11">
+        <v>23540.14789</v>
+      </c>
+      <c r="C11">
+        <v>4.47</v>
+      </c>
+      <c r="D11" t="s">
+        <v>478</v>
+      </c>
+      <c r="E11" t="s">
+        <v>478</v>
+      </c>
+      <c r="F11" t="s">
+        <v>478</v>
+      </c>
+      <c r="G11" t="s">
+        <v>478</v>
+      </c>
+      <c r="H11" t="s">
+        <v>478</v>
+      </c>
+      <c r="I11" t="s">
+        <v>478</v>
+      </c>
+      <c r="J11" t="s">
+        <v>478</v>
+      </c>
+      <c r="K11" t="s">
+        <v>478</v>
+      </c>
+      <c r="L11" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>1987</v>
+      </c>
+      <c r="B12">
+        <v>26310.234110000001</v>
+      </c>
+      <c r="C12">
+        <v>5.08</v>
+      </c>
+      <c r="D12">
+        <v>-3.3292177999999999E-2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>478</v>
+      </c>
+      <c r="F12" t="s">
+        <v>478</v>
+      </c>
+      <c r="G12" t="s">
+        <v>478</v>
+      </c>
+      <c r="H12" t="s">
+        <v>478</v>
+      </c>
+      <c r="I12" t="s">
+        <v>478</v>
+      </c>
+      <c r="J12" t="s">
+        <v>478</v>
+      </c>
+      <c r="K12" t="s">
+        <v>478</v>
+      </c>
+      <c r="L12" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1988</v>
+      </c>
+      <c r="B13">
+        <v>27358.8914</v>
+      </c>
+      <c r="C13">
+        <v>4.7699999999999996</v>
+      </c>
+      <c r="D13">
+        <v>1.2900270030000001</v>
+      </c>
+      <c r="E13" t="s">
+        <v>478</v>
+      </c>
+      <c r="F13" t="s">
+        <v>478</v>
+      </c>
+      <c r="G13" t="s">
+        <v>478</v>
+      </c>
+      <c r="H13" t="s">
+        <v>478</v>
+      </c>
+      <c r="I13" t="s">
+        <v>478</v>
+      </c>
+      <c r="J13" t="s">
+        <v>478</v>
+      </c>
+      <c r="K13" t="s">
+        <v>478</v>
+      </c>
+      <c r="L13" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>1989</v>
+      </c>
+      <c r="B14">
+        <v>25061.380980000002</v>
+      </c>
+      <c r="C14">
+        <v>3.61</v>
+      </c>
+      <c r="D14">
+        <v>1.049146213</v>
+      </c>
+      <c r="E14" t="s">
+        <v>478</v>
+      </c>
+      <c r="F14" t="s">
+        <v>478</v>
+      </c>
+      <c r="G14" t="s">
+        <v>478</v>
+      </c>
+      <c r="H14" t="s">
+        <v>478</v>
+      </c>
+      <c r="I14" t="s">
+        <v>478</v>
+      </c>
+      <c r="J14" t="s">
+        <v>478</v>
+      </c>
+      <c r="K14" t="s">
+        <v>478</v>
+      </c>
+      <c r="L14" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1990</v>
+      </c>
+      <c r="B15">
+        <v>23503.43187</v>
+      </c>
+      <c r="C15">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>1983</v>
-      </c>
-      <c r="B6">
-        <v>5.1100000000000003</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>1984</v>
-      </c>
-      <c r="B7">
-        <v>4.7300000000000004</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>1985</v>
-      </c>
-      <c r="B8">
+      <c r="D15">
+        <v>1.3385839669999999</v>
+      </c>
+      <c r="E15" t="s">
+        <v>478</v>
+      </c>
+      <c r="F15" t="s">
+        <v>478</v>
+      </c>
+      <c r="G15" t="s">
+        <v>478</v>
+      </c>
+      <c r="H15">
+        <v>1.3829039E-2</v>
+      </c>
+      <c r="I15" t="s">
+        <v>478</v>
+      </c>
+      <c r="J15" t="s">
+        <v>478</v>
+      </c>
+      <c r="K15" t="s">
+        <v>478</v>
+      </c>
+      <c r="L15" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>1991</v>
+      </c>
+      <c r="B16">
+        <v>26693.90984</v>
+      </c>
+      <c r="C16">
+        <v>3.7</v>
+      </c>
+      <c r="D16">
+        <v>0.170562924</v>
+      </c>
+      <c r="E16" t="s">
+        <v>478</v>
+      </c>
+      <c r="F16" t="s">
+        <v>478</v>
+      </c>
+      <c r="G16" t="s">
+        <v>478</v>
+      </c>
+      <c r="H16" t="s">
+        <v>478</v>
+      </c>
+      <c r="I16" t="s">
+        <v>478</v>
+      </c>
+      <c r="J16" t="s">
+        <v>478</v>
+      </c>
+      <c r="K16" t="s">
+        <v>478</v>
+      </c>
+      <c r="L16" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>1992</v>
+      </c>
+      <c r="B17">
+        <v>31204.025000000001</v>
+      </c>
+      <c r="C17">
         <v>4.57</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>1986</v>
-      </c>
-      <c r="B9">
-        <v>4.7300000000000004</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>1987</v>
-      </c>
-      <c r="B10">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>1988</v>
-      </c>
-      <c r="B11">
+      <c r="D17">
+        <v>2.041381119</v>
+      </c>
+      <c r="E17" t="s">
+        <v>478</v>
+      </c>
+      <c r="F17" t="s">
+        <v>478</v>
+      </c>
+      <c r="G17" t="s">
+        <v>478</v>
+      </c>
+      <c r="H17" t="s">
+        <v>478</v>
+      </c>
+      <c r="I17">
+        <v>137629</v>
+      </c>
+      <c r="J17" t="s">
+        <v>478</v>
+      </c>
+      <c r="K17" t="s">
+        <v>478</v>
+      </c>
+      <c r="L17" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>1993</v>
+      </c>
+      <c r="B18">
+        <v>29155.798309999998</v>
+      </c>
+      <c r="C18">
+        <v>4.2</v>
+      </c>
+      <c r="D18">
+        <v>2.6217975990000002</v>
+      </c>
+      <c r="E18">
+        <v>-34.07</v>
+      </c>
+      <c r="F18">
+        <v>-24.76</v>
+      </c>
+      <c r="G18" t="s">
+        <v>478</v>
+      </c>
+      <c r="H18">
+        <v>1.1566763000000001E-2</v>
+      </c>
+      <c r="I18">
+        <v>11826375</v>
+      </c>
+      <c r="J18" t="s">
+        <v>478</v>
+      </c>
+      <c r="K18" t="s">
+        <v>478</v>
+      </c>
+      <c r="L18">
+        <v>5.902497576</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>1994</v>
+      </c>
+      <c r="B19">
+        <v>26995.367300000002</v>
+      </c>
+      <c r="C19">
+        <v>4.1900000000000004</v>
+      </c>
+      <c r="D19">
+        <v>1.7883762050000001</v>
+      </c>
+      <c r="E19">
+        <v>-28.6</v>
+      </c>
+      <c r="F19">
+        <v>-34.590000000000003</v>
+      </c>
+      <c r="G19">
+        <v>3.09</v>
+      </c>
+      <c r="H19" t="s">
+        <v>478</v>
+      </c>
+      <c r="I19">
+        <v>3390830</v>
+      </c>
+      <c r="J19" t="s">
+        <v>478</v>
+      </c>
+      <c r="K19" t="s">
+        <v>478</v>
+      </c>
+      <c r="L19" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>1995</v>
+      </c>
+      <c r="B20">
+        <v>23078.352999999999</v>
+      </c>
+      <c r="C20">
+        <v>3.99</v>
+      </c>
+      <c r="D20">
+        <v>2.2971653760000001</v>
+      </c>
+      <c r="E20">
+        <v>-8.67</v>
+      </c>
+      <c r="F20">
+        <v>-40.36</v>
+      </c>
+      <c r="G20">
+        <v>3.0529999999999999</v>
+      </c>
+      <c r="H20" t="s">
+        <v>478</v>
+      </c>
+      <c r="I20">
+        <v>3788518</v>
+      </c>
+      <c r="J20" t="s">
+        <v>478</v>
+      </c>
+      <c r="K20" t="s">
+        <v>478</v>
+      </c>
+      <c r="L20" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>1996</v>
+      </c>
+      <c r="B21">
+        <v>24763.241699999999</v>
+      </c>
+      <c r="C21">
+        <v>4.32</v>
+      </c>
+      <c r="D21">
+        <v>3.1946072170000002</v>
+      </c>
+      <c r="E21">
+        <v>-23.51</v>
+      </c>
+      <c r="F21">
+        <v>-35.93</v>
+      </c>
+      <c r="G21">
+        <v>3.0310000000000001</v>
+      </c>
+      <c r="H21">
+        <v>4.24867E-4</v>
+      </c>
+      <c r="I21">
+        <v>11262967</v>
+      </c>
+      <c r="J21" t="s">
+        <v>478</v>
+      </c>
+      <c r="K21" t="s">
+        <v>478</v>
+      </c>
+      <c r="L21">
+        <v>5.5693833929999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>1997</v>
+      </c>
+      <c r="B22">
+        <v>28654.26125</v>
+      </c>
+      <c r="C22">
+        <v>4.0199999999999996</v>
+      </c>
+      <c r="D22">
+        <v>2.8368044889999999</v>
+      </c>
+      <c r="E22">
+        <v>-15.56</v>
+      </c>
+      <c r="F22">
+        <v>-30.68</v>
+      </c>
+      <c r="G22" t="s">
+        <v>478</v>
+      </c>
+      <c r="H22" t="s">
+        <v>478</v>
+      </c>
+      <c r="I22">
+        <v>4124667</v>
+      </c>
+      <c r="J22" t="s">
+        <v>478</v>
+      </c>
+      <c r="K22" t="s">
+        <v>478</v>
+      </c>
+      <c r="L22" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>1998</v>
+      </c>
+      <c r="B23">
+        <v>41169.819340000002</v>
+      </c>
+      <c r="C23">
+        <v>5.33</v>
+      </c>
+      <c r="D23">
+        <v>1.0035694129999999</v>
+      </c>
+      <c r="E23">
+        <v>44.75</v>
+      </c>
+      <c r="F23">
+        <v>-5</v>
+      </c>
+      <c r="G23">
+        <v>2.794</v>
+      </c>
+      <c r="H23" t="s">
+        <v>478</v>
+      </c>
+      <c r="I23">
+        <v>9035599</v>
+      </c>
+      <c r="J23" t="s">
+        <v>478</v>
+      </c>
+      <c r="K23" t="s">
+        <v>478</v>
+      </c>
+      <c r="L23" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>1999</v>
+      </c>
+      <c r="B24">
+        <v>41122.258750000001</v>
+      </c>
+      <c r="C24">
+        <v>3.51</v>
+      </c>
+      <c r="D24">
+        <v>1.7581501799999999</v>
+      </c>
+      <c r="E24">
+        <v>-1.33</v>
+      </c>
+      <c r="F24">
+        <v>-40.950000000000003</v>
+      </c>
+      <c r="G24">
+        <v>2.7040000000000002</v>
+      </c>
+      <c r="H24">
+        <v>-5.1038430000000003E-3</v>
+      </c>
+      <c r="I24">
+        <v>18492742</v>
+      </c>
+      <c r="J24" t="s">
+        <v>478</v>
+      </c>
+      <c r="K24" t="s">
+        <v>478</v>
+      </c>
+      <c r="L24">
+        <v>5.0962059379999998</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2000</v>
+      </c>
+      <c r="B25">
+        <v>47363.523549999998</v>
+      </c>
+      <c r="C25">
+        <v>4.22</v>
+      </c>
+      <c r="D25">
+        <v>0.88124960900000004</v>
+      </c>
+      <c r="E25">
+        <v>0.34</v>
+      </c>
+      <c r="F25">
+        <v>-30.52</v>
+      </c>
+      <c r="G25">
+        <v>3.177</v>
+      </c>
+      <c r="H25" t="s">
+        <v>478</v>
+      </c>
+      <c r="I25">
+        <v>22385837</v>
+      </c>
+      <c r="J25" t="s">
+        <v>478</v>
+      </c>
+      <c r="K25">
+        <v>1.57</v>
+      </c>
+      <c r="L25" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>2001</v>
+      </c>
+      <c r="B26">
+        <v>45288.103029999998</v>
+      </c>
+      <c r="C26">
+        <v>4.8600000000000003</v>
+      </c>
+      <c r="D26">
+        <v>1.550219064</v>
+      </c>
+      <c r="E26">
+        <v>16.91</v>
+      </c>
+      <c r="F26">
+        <v>-6.29</v>
+      </c>
+      <c r="G26">
+        <v>2.9209999999999998</v>
+      </c>
+      <c r="H26">
+        <v>2.3104279999999998E-3</v>
+      </c>
+      <c r="I26">
+        <v>19340020</v>
+      </c>
+      <c r="J26" t="s">
+        <v>478</v>
+      </c>
+      <c r="K26">
+        <v>1.7330000000000001</v>
+      </c>
+      <c r="L26">
+        <v>5.9022860359999996</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>2002</v>
+      </c>
+      <c r="B27">
+        <v>34955.136729999998</v>
+      </c>
+      <c r="C27">
+        <v>3.95</v>
+      </c>
+      <c r="D27">
+        <v>-0.35405105999999997</v>
+      </c>
+      <c r="E27">
+        <v>8.06</v>
+      </c>
+      <c r="F27">
+        <v>-18.16</v>
+      </c>
+      <c r="G27">
+        <v>2.6909999999999998</v>
+      </c>
+      <c r="H27" t="s">
+        <v>478</v>
+      </c>
+      <c r="I27">
+        <v>24663313</v>
+      </c>
+      <c r="J27" t="s">
+        <v>478</v>
+      </c>
+      <c r="K27" t="s">
+        <v>478</v>
+      </c>
+      <c r="L27" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>2003</v>
+      </c>
+      <c r="B28">
+        <v>31270.472610000001</v>
+      </c>
+      <c r="C28">
+        <v>5.52</v>
+      </c>
+      <c r="D28">
+        <v>-0.35632142</v>
+      </c>
+      <c r="E28">
+        <v>51.96</v>
+      </c>
+      <c r="F28">
+        <v>29.63</v>
+      </c>
+      <c r="G28">
+        <v>3.2069999999999999</v>
+      </c>
+      <c r="H28">
+        <v>2.3443919999999998E-3</v>
+      </c>
+      <c r="I28">
+        <v>12236933</v>
+      </c>
+      <c r="J28">
+        <v>200382.74129999999</v>
+      </c>
+      <c r="K28">
+        <v>1.6759999999999999</v>
+      </c>
+      <c r="L28">
+        <v>6.102874334</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>2004</v>
+      </c>
+      <c r="B29">
+        <v>31996.64934</v>
+      </c>
+      <c r="C29">
+        <v>4.38</v>
+      </c>
+      <c r="D29">
+        <v>2.7210139189999998</v>
+      </c>
+      <c r="E29">
+        <v>-10.87</v>
+      </c>
+      <c r="F29">
+        <v>36.78</v>
+      </c>
+      <c r="G29">
+        <v>2.8620000000000001</v>
+      </c>
+      <c r="H29" t="s">
+        <v>478</v>
+      </c>
+      <c r="I29">
+        <v>5060913</v>
+      </c>
+      <c r="J29" t="s">
+        <v>478</v>
+      </c>
+      <c r="K29" t="s">
+        <v>478</v>
+      </c>
+      <c r="L29" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>2005</v>
+      </c>
+      <c r="B30">
+        <v>37616.717830000001</v>
+      </c>
+      <c r="C30">
+        <v>4.5</v>
+      </c>
+      <c r="D30">
+        <v>1.6392317940000001</v>
+      </c>
+      <c r="E30">
+        <v>-20.77</v>
+      </c>
+      <c r="F30">
+        <v>44.84</v>
+      </c>
+      <c r="G30">
+        <v>3.1</v>
+      </c>
+      <c r="H30">
+        <v>-5.931057E-3</v>
+      </c>
+      <c r="I30">
+        <v>12723811</v>
+      </c>
+      <c r="J30">
+        <v>569076.51210000005</v>
+      </c>
+      <c r="K30">
+        <v>1.6120000000000001</v>
+      </c>
+      <c r="L30">
+        <v>5.8673143230000004</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>2006</v>
+      </c>
+      <c r="B31">
+        <v>38903.938900000001</v>
+      </c>
+      <c r="C31">
+        <v>4.18</v>
+      </c>
+      <c r="D31">
+        <v>1.8577682849999999</v>
+      </c>
+      <c r="E31">
+        <v>-11.29</v>
+      </c>
+      <c r="F31">
+        <v>-21.67</v>
+      </c>
+      <c r="G31">
+        <v>2.9609999999999999</v>
+      </c>
+      <c r="H31" t="s">
+        <v>478</v>
+      </c>
+      <c r="I31">
+        <v>4829656</v>
+      </c>
+      <c r="J31" t="s">
+        <v>478</v>
+      </c>
+      <c r="K31" t="s">
+        <v>478</v>
+      </c>
+      <c r="L31" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>2007</v>
+      </c>
+      <c r="B32">
+        <v>33777.368210000001</v>
+      </c>
+      <c r="C32">
+        <v>3.26</v>
+      </c>
+      <c r="D32">
+        <v>1.8475412170000001</v>
+      </c>
+      <c r="E32">
+        <v>-10.58</v>
+      </c>
+      <c r="F32">
+        <v>22.93</v>
+      </c>
+      <c r="G32">
+        <v>2.6960000000000002</v>
+      </c>
+      <c r="H32">
+        <v>-6.541926E-3</v>
+      </c>
+      <c r="I32">
+        <v>19115666</v>
+      </c>
+      <c r="J32" t="s">
+        <v>478</v>
+      </c>
+      <c r="K32">
+        <v>1.399</v>
+      </c>
+      <c r="L32">
+        <v>5.0703875089999997</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>2008</v>
+      </c>
+      <c r="B33">
+        <v>27815.09187</v>
+      </c>
+      <c r="C33">
+        <v>3.63</v>
+      </c>
+      <c r="D33">
+        <v>0.135563507</v>
+      </c>
+      <c r="E33">
+        <v>-10.08</v>
+      </c>
+      <c r="F33">
+        <v>31.03</v>
+      </c>
+      <c r="G33">
+        <v>2.92</v>
+      </c>
+      <c r="H33" t="s">
+        <v>478</v>
+      </c>
+      <c r="I33">
+        <v>5386141</v>
+      </c>
+      <c r="J33" t="s">
+        <v>478</v>
+      </c>
+      <c r="K33" t="s">
+        <v>478</v>
+      </c>
+      <c r="L33" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>2009</v>
+      </c>
+      <c r="B34">
+        <v>20555.143349999998</v>
+      </c>
+      <c r="C34">
+        <v>3.29</v>
+      </c>
+      <c r="D34">
+        <v>-0.58334247400000006</v>
+      </c>
+      <c r="E34">
+        <v>-31.22</v>
+      </c>
+      <c r="F34">
+        <v>-34.24</v>
+      </c>
+      <c r="G34">
+        <v>2.867</v>
+      </c>
+      <c r="H34">
+        <v>-4.9044259999999999E-3</v>
+      </c>
+      <c r="I34">
+        <v>6663248</v>
+      </c>
+      <c r="J34" t="s">
+        <v>478</v>
+      </c>
+      <c r="K34">
+        <v>1.296</v>
+      </c>
+      <c r="L34">
+        <v>4.9795084379999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>2010</v>
+      </c>
+      <c r="B35">
+        <v>21421.645489999999</v>
+      </c>
+      <c r="C35">
+        <v>4.59</v>
+      </c>
+      <c r="D35">
+        <v>-0.94295863300000005</v>
+      </c>
+      <c r="E35">
+        <v>19.059999999999999</v>
+      </c>
+      <c r="F35">
+        <v>-2.21</v>
+      </c>
+      <c r="G35">
+        <v>3.26</v>
+      </c>
+      <c r="H35" t="s">
+        <v>478</v>
+      </c>
+      <c r="I35">
+        <v>1560332</v>
+      </c>
+      <c r="J35" t="s">
+        <v>478</v>
+      </c>
+      <c r="K35" t="s">
+        <v>478</v>
+      </c>
+      <c r="L35" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>2011</v>
+      </c>
+      <c r="B36">
+        <v>19328.910479999999</v>
+      </c>
+      <c r="C36">
+        <v>4.05</v>
+      </c>
+      <c r="D36">
+        <v>1.6338793030000001</v>
+      </c>
+      <c r="E36">
+        <v>65.7</v>
+      </c>
+      <c r="F36">
+        <v>58.15</v>
+      </c>
+      <c r="G36">
+        <v>2.7480000000000002</v>
+      </c>
+      <c r="H36">
+        <v>-5.3047739999999999E-3</v>
+      </c>
+      <c r="I36">
+        <v>5163167</v>
+      </c>
+      <c r="J36">
+        <v>620474.25989999995</v>
+      </c>
+      <c r="K36" t="s">
+        <v>478</v>
+      </c>
+      <c r="L36">
+        <v>5.4603732559999996</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>2012</v>
+      </c>
+      <c r="B37">
+        <v>20208.851989999999</v>
+      </c>
+      <c r="C37">
+        <v>3.33</v>
+      </c>
+      <c r="D37" t="s">
+        <v>478</v>
+      </c>
+      <c r="E37">
+        <v>-11.88</v>
+      </c>
+      <c r="F37">
+        <v>29.63</v>
+      </c>
+      <c r="G37" t="s">
+        <v>478</v>
+      </c>
+      <c r="H37" t="s">
+        <v>478</v>
+      </c>
+      <c r="I37">
+        <v>5606338</v>
+      </c>
+      <c r="J37" t="s">
+        <v>478</v>
+      </c>
+      <c r="K37" t="s">
+        <v>478</v>
+      </c>
+      <c r="L37" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>2013</v>
+      </c>
+      <c r="B38">
+        <v>20384.51312</v>
+      </c>
+      <c r="C38">
+        <v>3.99</v>
+      </c>
+      <c r="D38">
+        <v>0.77391578100000002</v>
+      </c>
+      <c r="E38">
+        <v>-2.8</v>
+      </c>
+      <c r="F38">
+        <v>47.85</v>
+      </c>
+      <c r="G38">
+        <v>3.2879999999999998</v>
+      </c>
+      <c r="H38">
+        <v>3.0496880000000001E-3</v>
+      </c>
+      <c r="I38">
+        <v>12541222</v>
+      </c>
+      <c r="J38">
+        <v>460745.71909999999</v>
+      </c>
+      <c r="K38">
+        <v>0.96499999999999997</v>
+      </c>
+      <c r="L38">
+        <v>5.3840517229999998</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>2014</v>
+      </c>
+      <c r="B39">
+        <v>15213.646629999999</v>
+      </c>
+      <c r="C39">
+        <v>4.3600000000000003</v>
+      </c>
+      <c r="D39" t="s">
+        <v>478</v>
+      </c>
+      <c r="E39">
+        <v>-7.28</v>
+      </c>
+      <c r="F39">
+        <v>-21.66</v>
+      </c>
+      <c r="G39" t="s">
+        <v>478</v>
+      </c>
+      <c r="H39" t="s">
+        <v>478</v>
+      </c>
+      <c r="I39">
+        <v>22022421</v>
+      </c>
+      <c r="J39" t="s">
+        <v>478</v>
+      </c>
+      <c r="K39" t="s">
+        <v>478</v>
+      </c>
+      <c r="L39" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>2015</v>
+      </c>
+      <c r="B40">
+        <v>16698.362219999999</v>
+      </c>
+      <c r="C40">
+        <v>5.36</v>
+      </c>
+      <c r="D40">
+        <v>0.357685423</v>
+      </c>
+      <c r="E40">
+        <v>14.24</v>
+      </c>
+      <c r="F40">
+        <v>25.12</v>
+      </c>
+      <c r="G40">
+        <v>3.3370000000000002</v>
+      </c>
+      <c r="H40">
+        <v>-2.7227940000000002E-3</v>
+      </c>
+      <c r="I40">
+        <v>3607343</v>
+      </c>
+      <c r="J40">
+        <v>436759.00150000001</v>
+      </c>
+      <c r="K40">
+        <v>1.302</v>
+      </c>
+      <c r="L40">
+        <v>6.3322652210000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>2016</v>
+      </c>
+      <c r="B41">
+        <v>17842.354159999999</v>
+      </c>
+      <c r="C41">
+        <v>5.81</v>
+      </c>
+      <c r="D41" t="s">
+        <v>478</v>
+      </c>
+      <c r="E41">
+        <v>19.23</v>
+      </c>
+      <c r="F41">
+        <v>36.64</v>
+      </c>
+      <c r="G41" t="s">
+        <v>478</v>
+      </c>
+      <c r="H41" t="s">
+        <v>478</v>
+      </c>
+      <c r="I41">
+        <v>3652619</v>
+      </c>
+      <c r="J41" t="s">
+        <v>478</v>
+      </c>
+      <c r="K41" t="s">
+        <v>478</v>
+      </c>
+      <c r="L41" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>2017</v>
+      </c>
+      <c r="B42">
+        <v>19040.17513</v>
+      </c>
+      <c r="C42">
+        <v>4.75</v>
+      </c>
+      <c r="D42">
+        <v>1.481673655</v>
+      </c>
+      <c r="E42">
+        <v>11.32</v>
+      </c>
+      <c r="F42">
+        <v>-28.81</v>
+      </c>
+      <c r="G42">
+        <v>3.2890000000000001</v>
+      </c>
+      <c r="H42">
+        <v>-7.7513720000000003E-3</v>
+      </c>
+      <c r="I42">
+        <v>12439171</v>
+      </c>
+      <c r="J42">
+        <v>203106.8254</v>
+      </c>
+      <c r="K42">
+        <v>1.1319999999999999</v>
+      </c>
+      <c r="L42">
+        <v>5.8954712049999998</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>2018</v>
+      </c>
+      <c r="B43">
+        <v>23418.206750000001</v>
+      </c>
+      <c r="C43">
         <v>4.7</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>1989</v>
-      </c>
-      <c r="B12">
-        <v>4.05</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>1990</v>
-      </c>
-      <c r="B13">
-        <v>4.12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>1991</v>
-      </c>
-      <c r="B14">
-        <v>4.38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>1992</v>
-      </c>
-      <c r="B15">
-        <v>4.8899999999999997</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>1993</v>
-      </c>
-      <c r="B16">
-        <v>4.5199999999999996</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>1994</v>
-      </c>
-      <c r="B17">
-        <v>4.47</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>1995</v>
-      </c>
-      <c r="B18">
-        <v>4.04</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>1996</v>
-      </c>
-      <c r="B19">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>1997</v>
-      </c>
-      <c r="B20">
-        <v>4.5599999999999996</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>1998</v>
-      </c>
-      <c r="B21">
-        <v>5.73</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>1999</v>
-      </c>
-      <c r="B22">
-        <v>4.43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>2000</v>
-      </c>
-      <c r="B23">
-        <v>4.51</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>2001</v>
-      </c>
-      <c r="B24">
-        <v>4.9800000000000004</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>2002</v>
-      </c>
-      <c r="B25">
-        <v>4.2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>2003</v>
-      </c>
-      <c r="B26">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27">
-        <v>2004</v>
-      </c>
-      <c r="B27">
-        <v>4.5999999999999996</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28">
-        <v>2005</v>
-      </c>
-      <c r="B28">
-        <v>4.91</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29">
-        <v>2006</v>
-      </c>
-      <c r="B29">
-        <v>4.63</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30">
-        <v>2007</v>
-      </c>
-      <c r="B30">
-        <v>4.13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31">
-        <v>2008</v>
-      </c>
-      <c r="B31">
-        <v>4.33</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32">
-        <v>2009</v>
-      </c>
-      <c r="B32">
-        <v>3.66</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33">
-        <v>2010</v>
-      </c>
-      <c r="B33">
-        <v>5.21</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34">
-        <v>2011</v>
-      </c>
-      <c r="B34">
-        <v>4.55</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35">
-        <v>2012</v>
-      </c>
-      <c r="B35">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36">
-        <v>2013</v>
-      </c>
-      <c r="B36">
-        <v>4.18</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37">
-        <v>2014</v>
-      </c>
-      <c r="B37">
-        <v>4.7300000000000004</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38">
-        <v>2015</v>
-      </c>
-      <c r="B38">
-        <v>5.88</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39">
-        <v>2016</v>
-      </c>
-      <c r="B39">
-        <v>5.71</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40">
-        <v>2017</v>
-      </c>
-      <c r="B40">
-        <v>4.75</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41">
-        <v>2018</v>
-      </c>
-      <c r="B41">
-        <v>5.0999999999999996</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42">
+      <c r="D43" t="s">
+        <v>478</v>
+      </c>
+      <c r="E43">
+        <v>26.34</v>
+      </c>
+      <c r="F43">
+        <v>-31.62</v>
+      </c>
+      <c r="G43" t="s">
+        <v>478</v>
+      </c>
+      <c r="H43" t="s">
+        <v>478</v>
+      </c>
+      <c r="I43">
+        <v>8283740</v>
+      </c>
+      <c r="J43" t="s">
+        <v>478</v>
+      </c>
+      <c r="K43" t="s">
+        <v>478</v>
+      </c>
+      <c r="L43" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A44">
         <v>2019</v>
       </c>
-      <c r="B42">
-        <v>5.94</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43">
+      <c r="B44">
+        <v>23642.562190000001</v>
+      </c>
+      <c r="C44">
+        <v>5.62</v>
+      </c>
+      <c r="D44">
+        <v>-0.172489369</v>
+      </c>
+      <c r="E44">
+        <v>5.46</v>
+      </c>
+      <c r="F44">
+        <v>-10.67</v>
+      </c>
+      <c r="G44">
+        <v>3.3559999999999999</v>
+      </c>
+      <c r="H44">
+        <v>4.349693E-3</v>
+      </c>
+      <c r="I44">
+        <v>10544652</v>
+      </c>
+      <c r="J44">
+        <v>336170</v>
+      </c>
+      <c r="K44">
+        <v>1.4970000000000001</v>
+      </c>
+      <c r="L44">
+        <v>6.3910258850000004</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A45">
         <v>2020</v>
       </c>
-      <c r="B43">
-        <v>4.3</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44">
+      <c r="B45">
+        <v>19194.74266</v>
+      </c>
+      <c r="C45">
+        <v>4.2300000000000004</v>
+      </c>
+      <c r="D45" t="s">
+        <v>478</v>
+      </c>
+      <c r="E45">
+        <v>-40.39</v>
+      </c>
+      <c r="F45">
+        <v>17.510000000000002</v>
+      </c>
+      <c r="G45" t="s">
+        <v>478</v>
+      </c>
+      <c r="H45" t="s">
+        <v>478</v>
+      </c>
+      <c r="I45">
+        <v>6933691</v>
+      </c>
+      <c r="J45" t="s">
+        <v>478</v>
+      </c>
+      <c r="K45" t="s">
+        <v>478</v>
+      </c>
+      <c r="L45" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A46">
         <v>2021</v>
       </c>
-      <c r="B44">
-        <v>4.26</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45">
+      <c r="B46">
+        <v>17110.174879999999</v>
+      </c>
+      <c r="C46">
+        <v>4.53</v>
+      </c>
+      <c r="D46">
+        <v>1.235706875</v>
+      </c>
+      <c r="E46">
+        <v>-6.82</v>
+      </c>
+      <c r="F46">
+        <v>44.66</v>
+      </c>
+      <c r="G46">
+        <v>3.1429999999999998</v>
+      </c>
+      <c r="H46">
+        <v>3.10428E-5</v>
+      </c>
+      <c r="I46">
+        <v>3500029</v>
+      </c>
+      <c r="J46" t="s">
+        <v>478</v>
+      </c>
+      <c r="K46" t="s">
+        <v>478</v>
+      </c>
+      <c r="L46">
+        <v>5.7438771109999998</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A47">
         <v>2022</v>
       </c>
-      <c r="B45">
-        <v>5.09</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46">
+      <c r="B47">
+        <v>19188.285739999999</v>
+      </c>
+      <c r="C47">
+        <v>4.32</v>
+      </c>
+      <c r="D47" t="s">
+        <v>478</v>
+      </c>
+      <c r="E47">
+        <v>-7.79</v>
+      </c>
+      <c r="F47">
+        <v>-9.86</v>
+      </c>
+      <c r="G47" t="s">
+        <v>478</v>
+      </c>
+      <c r="H47" t="s">
+        <v>478</v>
+      </c>
+      <c r="I47">
+        <v>2551866</v>
+      </c>
+      <c r="J47" t="s">
+        <v>478</v>
+      </c>
+      <c r="K47" t="s">
+        <v>478</v>
+      </c>
+      <c r="L47" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A48">
         <v>2023</v>
       </c>
-      <c r="B46">
-        <v>4.4400000000000004</v>
+      <c r="B48">
+        <v>18865.697230000002</v>
+      </c>
+      <c r="C48">
+        <v>4.22</v>
+      </c>
+      <c r="D48">
+        <v>1.741747624</v>
+      </c>
+      <c r="E48">
+        <v>-12.28</v>
+      </c>
+      <c r="F48">
+        <v>-27.3</v>
+      </c>
+      <c r="G48">
+        <v>3.0110000000000001</v>
+      </c>
+      <c r="H48">
+        <v>9.2136499999999994E-5</v>
+      </c>
+      <c r="I48">
+        <v>4085143</v>
+      </c>
+      <c r="J48" t="s">
+        <v>478</v>
+      </c>
+      <c r="K48">
+        <v>1.677</v>
+      </c>
+      <c r="L48">
+        <v>5.477908824</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>2024</v>
+      </c>
+      <c r="B49">
+        <v>20266.09302</v>
+      </c>
+      <c r="C49">
+        <v>4.54</v>
+      </c>
+      <c r="D49" t="s">
+        <v>478</v>
+      </c>
+      <c r="E49">
+        <v>15.53</v>
+      </c>
+      <c r="F49">
+        <v>48.45</v>
+      </c>
+      <c r="G49" t="s">
+        <v>478</v>
+      </c>
+      <c r="H49" t="s">
+        <v>478</v>
+      </c>
+      <c r="I49">
+        <v>2066137</v>
+      </c>
+      <c r="J49" t="s">
+        <v>478</v>
+      </c>
+      <c r="K49" t="s">
+        <v>478</v>
+      </c>
+      <c r="L49" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>2025</v>
+      </c>
+      <c r="B50">
+        <v>20973.38492</v>
+      </c>
+      <c r="C50">
+        <v>5.16</v>
+      </c>
+      <c r="D50">
+        <v>-1.6934433</v>
+      </c>
+      <c r="E50">
+        <v>-3.38</v>
+      </c>
+      <c r="F50">
+        <v>-23.61</v>
+      </c>
+      <c r="G50" t="s">
+        <v>478</v>
+      </c>
+      <c r="H50">
+        <v>-2.0086099999999999E-4</v>
+      </c>
+      <c r="I50">
+        <v>3698795</v>
+      </c>
+      <c r="J50" t="s">
+        <v>478</v>
+      </c>
+      <c r="K50" t="s">
+        <v>478</v>
+      </c>
+      <c r="L50">
+        <v>6.1345535269999996</v>
       </c>
     </row>
   </sheetData>
@@ -5750,10 +7312,10 @@
         <v>303</v>
       </c>
       <c r="Y1" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>481</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>482</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>468</v>
@@ -5937,22 +7499,22 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>483</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>487</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>488</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>153</v>
@@ -5961,7 +7523,7 @@
         <v>162</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated scripts and output and ran projections
</commit_message>
<xml_diff>
--- a/2026/data/GOA_arrowtooth_2026.xlsx
+++ b/2026/data/GOA_arrowtooth_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kalei.shotwell\Work\GitHub\GOA-ATF-ESP\2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7178123F-A3A1-40A7-B288-8A1EC230E66A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB61D98-EFB9-49B9-A0FB-2F05349C94E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2568" yWindow="1920" windowWidth="26136" windowHeight="13704" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31596" yWindow="744" windowWidth="26136" windowHeight="13704" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data" sheetId="1" r:id="rId1"/>
@@ -59121,7 +59121,7 @@
         <v>0</v>
       </c>
       <c r="AA2">
-        <v>1</v>
+        <v>0.1188226</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
@@ -59186,7 +59186,7 @@
         <v>0</v>
       </c>
       <c r="AA3">
-        <v>0.1188226</v>
+        <v>0.1173554</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">

</xml_diff>